<commit_message>
added Comparison_to_other_tools to Table_EV1
</commit_message>
<xml_diff>
--- a/Table_EV1.xlsx
+++ b/Table_EV1.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Resource_Level" sheetId="4" r:id="rId4"/>
     <sheet name="Set_Level" sheetId="5" r:id="rId5"/>
     <sheet name="Term_Size_Distribution" sheetId="6" r:id="rId6"/>
+    <sheet name="Comparison_to_other_tools" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -356,7 +357,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -458,6 +459,23 @@
       <c r="C6" t="inlineStr">
         <is>
           <t>Target membership composition across 1 term, 2 terms, and &gt;2 terms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sheet 6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>MetaProViz comparison to other tools.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Comparison to MetaboAnalyst R 4.0.</t>
         </is>
       </c>
     </row>
@@ -3499,4 +3517,322 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>MetaProViz</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>MetaboAnalyst R 4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Workflow scope</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>End-to-end metabolomics workflow</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>✔ Modular workflow integrating processing, analysis, and interpretation</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>✔ Comprehensive workflows covering multiple analysis types with strong web-based focus</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Data integration</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Exometabolomics (consumption/release) analysis</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>✔ Dedicated workflows linking intra- and extracellular metabolite changes</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>◯ No dedicated workflows explicitly described in available documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Prior knowledge integration</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>General prior knowledge usage</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>✔ Integrated across multiple steps of analysis</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>✔ Primarily used for pathway/enrichment analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Prior knowledge integration</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Metabolite identifier (ID) translation</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>✔ Systematic translation across databases with annotation expansion</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>✔ ID mapping supported</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Prior knowledge integration</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ID ambiguity quantification</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>✔ Explicit assessment and reporting of mapping ambiguities</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>◯ Not explicitly described</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Prior knowledge integration</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Gene → metabolite set conversion</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>✔ Reaction-based conversion using metabolic networks (e.g. Recon3D/COSMOS)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>◯ Not explicitly described</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Prior knowledge integration</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Receptor/transporter integration</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>✔ Included via curated resources (e.g. MetalinksDB)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>◯ Limited or not explicitly described</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Functional analysis</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Classical enrichment analysis</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Functional analysis</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Multi-condition / biologically informed clustering</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>✔ Implemented</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>◯ Limited or not explicitly described</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Functional analysis</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Integration with exometabolomics data</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>✔ Direct integration into functional analysis</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>◯ Not explicitly described</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Usability &amp; implementation</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Reproducible workflows</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>✔ Scriptable, log-based workflows in R/Bioconductor</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>✔ Available R package, Package dependencies need to be installed separatly</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Usability &amp; implementation</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>User guidance / automated checks</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>✔ Integrated messages, logging, and statistical guidance</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>◯ Limited or not explicitly described</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Usability &amp; implementation</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Interface focus</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>✔ Scriptable, workflow-oriented (Bioconductor ecosystem)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>✔ Strong focus on web-based accessibility</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>